<commit_message>
Correct CBAM flag on tin boxes: not applicable, Y824 code required instead
Per TARIC for 7310 21 90 00 only document code Y824 applies (Art. 3g
of Regulation (EU) 833/2014 — proof of no Russian iron/steel inputs),
not CBAM. Note added to request a non-Russian-origin steel declaration
from the supplier.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014CE6n4KCaiUV6ip7PuLiEs
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Angry_Beards_3810.xlsx
+++ b/output/HS_Code_Summary_Angry_Beards_3810.xlsx
@@ -534,7 +534,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>CBAM</t>
+          <t>CBAM / Y824</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -602,7 +602,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>ANO — kap. 7310 (železo/ocel), Annex I</t>
+          <t>NE — pouze kód Y824</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -654,7 +654,7 @@
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>⚠ CBAM: plechovky (číslo 7310, železo/ocel) spadají pod CBAM Annex I — vzniká ohlašovací povinnost CBAM.</t>
+          <t>⚠ Plechovky (7310 21 90 00): CBAM se dle TARIC neuplatňuje — vyžaduje se pouze kód Y824 (čl. 3g nařízení (EU) č. 833/2014, sankce vůči Rusku): doklad, že při zpracování ve třetí zemi nebyly použity železo/ocel ruského původu. Od dodavatele vyžádat prohlášení / mill test certificate.</t>
         </is>
       </c>
       <c r="B11" s="12" t="n"/>

</xml_diff>